<commit_message>
Add 30 sources and 1 QA Rules exception to defence source universe
Appends 12 global prime contractors (as named exceptions to the
Australian-HQ rule), 2 government agencies filling named coverage
gaps (critical minerals, export controls), 2 Tasmanian companies
(Incat, Liferaft), 3 export/finance bodies (Team Defence Australia,
EFA, NRFC), 2 ASX-listed additions (XTEK, AVA Risk), 6 X/Twitter
accounts for ministerial and agency channels, and 3 media outlets
(The Nightly, AAP, Sky News). All rows marked NEEDS VERIFICATION.

QA Rules sheet gains a named-exception entry documenting the 12
offshore-parented primes approved to bypass Rule 2.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/australian_defence_source_universe.xlsx
+++ b/data/australian_defence_source_universe.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z151"/>
+  <dimension ref="A1:Z181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -17471,6 +17471,3381 @@
       <c r="Z151" t="inlineStr">
         <is>
           <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Lockheed Martin Australia</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>GWEO, guided weapons, air and missile defence, C4ISR</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>https://www.lockheedmartin.com/en-au/index.html</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>US-parented (Lockheed Martin Corporation)</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>GWEO, guided weapons, air and missile defence, C4ISR</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R152" t="n">
+        <v>5</v>
+      </c>
+      <c r="S152" t="n">
+        <v>5</v>
+      </c>
+      <c r="T152" t="n">
+        <v>2</v>
+      </c>
+      <c r="U152" t="n">
+        <v>1</v>
+      </c>
+      <c r="V152" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W152" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X152" t="inlineStr">
+        <is>
+          <t>Prime contractor across GWEO, guided weapons and air/missile defence; frequently first to announce major program milestones and sovereign manufacturing investment.</t>
+        </is>
+      </c>
+      <c r="Y152" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z152" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Boeing Defence Australia</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Uncrewed systems (MQ-28 Ghost Bat), airpower, sustainment</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>QLD</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>https://www.boeing.com.au/</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>US-parented (The Boeing Company)</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>Uncrewed systems (MQ-28 Ghost Bat), airpower, sustainment</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R153" t="n">
+        <v>5</v>
+      </c>
+      <c r="S153" t="n">
+        <v>5</v>
+      </c>
+      <c r="T153" t="n">
+        <v>2</v>
+      </c>
+      <c r="U153" t="n">
+        <v>1</v>
+      </c>
+      <c r="V153" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W153" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X153" t="inlineStr">
+        <is>
+          <t>Leads MQ-28 Ghost Bat development locally; major airpower sustainment prime; announcements often precede official Defence releases.</t>
+        </is>
+      </c>
+      <c r="Y153" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z153" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>BAE Systems Australia</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Hunter class frigate, land systems, cyber</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>VIC</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>https://www.baesystems.com/en-aus/our-company/baes-australia</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>UK-parented (BAE Systems plc)</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>Hunter class frigate, land systems, cyber</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R154" t="n">
+        <v>5</v>
+      </c>
+      <c r="S154" t="n">
+        <v>5</v>
+      </c>
+      <c r="T154" t="n">
+        <v>2</v>
+      </c>
+      <c r="U154" t="n">
+        <v>1</v>
+      </c>
+      <c r="V154" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W154" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X154" t="inlineStr">
+        <is>
+          <t>Builds the Hunter class frigate program; one of the largest single defence industrial workforces in Australia.</t>
+        </is>
+      </c>
+      <c r="Y154" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z154" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Thales Australia</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Munitions (Benalla/Lithgow), sonar, protected vehicles</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>https://www.thalesgroup.com/en/countries/asia-pacific/australia</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>French-parented (Thales Group)</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>Munitions (Benalla/Lithgow), sonar, protected vehicles</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R155" t="n">
+        <v>5</v>
+      </c>
+      <c r="S155" t="n">
+        <v>5</v>
+      </c>
+      <c r="T155" t="n">
+        <v>2</v>
+      </c>
+      <c r="U155" t="n">
+        <v>1</v>
+      </c>
+      <c r="V155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X155" t="inlineStr">
+        <is>
+          <t>Operates sovereign munitions and weapons manufacturing; regular first-party source on capacity expansion and GWEO-adjacent contracts.</t>
+        </is>
+      </c>
+      <c r="Y155" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z155" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Rheinmetall Defence Australia</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Land 400 Boxer CRV, military vehicle manufacturing</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>QLD</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall-defence.com.au/</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>German-parented (Rheinmetall AG)</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>Land 400 Boxer CRV, military vehicle manufacturing</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R156" t="n">
+        <v>5</v>
+      </c>
+      <c r="S156" t="n">
+        <v>5</v>
+      </c>
+      <c r="T156" t="n">
+        <v>2</v>
+      </c>
+      <c r="U156" t="n">
+        <v>1</v>
+      </c>
+      <c r="V156" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W156" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X156" t="inlineStr">
+        <is>
+          <t>Leads Boxer CRV under Land 400 Phase 2; Military Vehicle Centre of Excellence is a flagship sovereign manufacturing case study.</t>
+        </is>
+      </c>
+      <c r="Y156" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z156" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Saab Australia</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Combat management systems, naval systems</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>https://www.saab.com/markets/australia</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>Swedish-parented (Saab AB)</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>Combat management systems, naval systems</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R157" t="n">
+        <v>5</v>
+      </c>
+      <c r="S157" t="n">
+        <v>5</v>
+      </c>
+      <c r="T157" t="n">
+        <v>2</v>
+      </c>
+      <c r="U157" t="n">
+        <v>1</v>
+      </c>
+      <c r="V157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X157" t="inlineStr">
+        <is>
+          <t>Supplies combat management systems across the surface fleet; material to naval capability announcements.</t>
+        </is>
+      </c>
+      <c r="Y157" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z157" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Elbit Systems of Australia</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Battle Management Systems, C4I, soldier systems</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>https://elbitsystems.com.au/</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>Israeli-parented (Elbit Systems Ltd)</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>Battle Management Systems, C4I, soldier systems</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R158" t="n">
+        <v>5</v>
+      </c>
+      <c r="S158" t="n">
+        <v>5</v>
+      </c>
+      <c r="T158" t="n">
+        <v>2</v>
+      </c>
+      <c r="U158" t="n">
+        <v>1</v>
+      </c>
+      <c r="V158" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W158" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X158" t="inlineStr">
+        <is>
+          <t>Delivers Army Battle Management System; relevant to land force digitisation announcements.</t>
+        </is>
+      </c>
+      <c r="Y158" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z158" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Leidos Australia</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Systems integration, sustainment, cyber</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>https://www.leidos.com/company/international/australia</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>US-parented (Leidos Holdings)</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>Systems integration, sustainment, cyber</t>
+        </is>
+      </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R159" t="n">
+        <v>5</v>
+      </c>
+      <c r="S159" t="n">
+        <v>5</v>
+      </c>
+      <c r="T159" t="n">
+        <v>2</v>
+      </c>
+      <c r="U159" t="n">
+        <v>1</v>
+      </c>
+      <c r="V159" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W159" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X159" t="inlineStr">
+        <is>
+          <t>Major systems integration and sustainment prime across multiple domains.</t>
+        </is>
+      </c>
+      <c r="Y159" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z159" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Raytheon Australia</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Air and missile defence, guided weapons</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>https://www.rtx.com/raytheon/who-we-are/global-locations/australia</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>US-parented (RTX Corporation)</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>Air and missile defence, guided weapons</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R160" t="n">
+        <v>5</v>
+      </c>
+      <c r="S160" t="n">
+        <v>5</v>
+      </c>
+      <c r="T160" t="n">
+        <v>2</v>
+      </c>
+      <c r="U160" t="n">
+        <v>1</v>
+      </c>
+      <c r="V160" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W160" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X160" t="inlineStr">
+        <is>
+          <t>Delivers air and missile defence and guided weapons capability; relevant to GWEO and NASAMS-related announcements.</t>
+        </is>
+      </c>
+      <c r="Y160" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z160" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Babcock Australasia</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Naval and aviation sustainment</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>https://www.babcock.com.au/</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>UK-parented (Babcock International Group)</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>Naval and aviation sustainment</t>
+        </is>
+      </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R161" t="n">
+        <v>5</v>
+      </c>
+      <c r="S161" t="n">
+        <v>5</v>
+      </c>
+      <c r="T161" t="n">
+        <v>2</v>
+      </c>
+      <c r="U161" t="n">
+        <v>1</v>
+      </c>
+      <c r="V161" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W161" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X161" t="inlineStr">
+        <is>
+          <t>Major sustainment prime across naval and aviation platforms.</t>
+        </is>
+      </c>
+      <c r="Y161" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z161" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>General Dynamics Land Systems - Australia</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Land 400 Phase 3 Redback IFV</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>QLD</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>https://www.gdlscanada.com/en/redback.html</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>US-parented (General Dynamics Corporation)</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>Land 400 Phase 3 Redback IFV</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R162" t="n">
+        <v>5</v>
+      </c>
+      <c r="S162" t="n">
+        <v>5</v>
+      </c>
+      <c r="T162" t="n">
+        <v>2</v>
+      </c>
+      <c r="U162" t="n">
+        <v>1</v>
+      </c>
+      <c r="V162" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W162" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X162" t="inlineStr">
+        <is>
+          <t>Delivers Redback IFV under Land 400 Phase 3, a top-tier land capability program.</t>
+        </is>
+      </c>
+      <c r="Y162" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z162" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Naval Group Australia</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Submarine industrial base, AUKUS transition support</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>https://www.naval-group.com/en/australia</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>French-parented (Naval Group)</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>Tier-1 global prime with a substantial Australian sovereign program; excluded under current QA Rule 2 (Australian-headquartered only) but material to contracts and market-moves reporting.</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>Submarine industrial base, AUKUS transition support</t>
+        </is>
+      </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R163" t="n">
+        <v>5</v>
+      </c>
+      <c r="S163" t="n">
+        <v>5</v>
+      </c>
+      <c r="T163" t="n">
+        <v>2</v>
+      </c>
+      <c r="U163" t="n">
+        <v>1</v>
+      </c>
+      <c r="V163" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W163" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X163" t="inlineStr">
+        <is>
+          <t>Retains a residual but relevant industrial and workforce role through the Attack class transition to AUKUS; useful for continuity and contract wind-down reporting.</t>
+        </is>
+      </c>
+      <c r="Y163" t="inlineStr">
+        <is>
+          <t>ADDED AS NAMED EXCEPTION to QA Rule 2 - see QA Rules sheet update. Verify current AU newsroom/press-release URL before activating.</t>
+        </is>
+      </c>
+      <c r="Z163" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Critical Minerals Facilitation Office</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Adjacent Domain</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Critical Minerals</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Commonwealth agency</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>https://www.industry.gov.au/science-technology-and-innovation/critical-minerals</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>Australian Government</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>No source in the universe currently covers critical minerals, despite it being a named category in the Email Logic template (Section 5).</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>Critical minerals, sovereign supply chains, processing investment</t>
+        </is>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R164" t="n">
+        <v>4</v>
+      </c>
+      <c r="S164" t="n">
+        <v>4</v>
+      </c>
+      <c r="T164" t="n">
+        <v>2</v>
+      </c>
+      <c r="U164" t="n">
+        <v>2</v>
+      </c>
+      <c r="V164" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W164" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X164" t="inlineStr">
+        <is>
+          <t>Fills a named coverage gap (critical minerals) with zero prior representation in the source list.</t>
+        </is>
+      </c>
+      <c r="Y164" t="inlineStr">
+        <is>
+          <t>VERIFY exact URL - office structure/URL may have changed.</t>
+        </is>
+      </c>
+      <c r="Z164" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Defence Export Controls</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Export Controls</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Commonwealth agency</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>https://www.defence.gov.au/business-industry/export</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>Australian Government</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>Export controls is a named escalation trigger in Collection Logic Step 7 but has no dedicated source.</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>Defence and Strategic Goods List (DSGL), defence trade controls, export permits</t>
+        </is>
+      </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="R165" t="n">
+        <v>4</v>
+      </c>
+      <c r="S165" t="n">
+        <v>4</v>
+      </c>
+      <c r="T165" t="n">
+        <v>2</v>
+      </c>
+      <c r="U165" t="n">
+        <v>2</v>
+      </c>
+      <c r="V165" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W165" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X165" t="inlineStr">
+        <is>
+          <t>Direct source for export-control actions and DSGL changes rather than relying on incidental mentions in general Defence releases.</t>
+        </is>
+      </c>
+      <c r="Y165" t="inlineStr">
+        <is>
+          <t>VERIFY exact URL and page structure.</t>
+        </is>
+      </c>
+      <c r="Z165" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Incat Tasmania</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Maritime, high-speed vessels</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>TAS</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>https://www.incat.com.au/</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>Only Tasmania-headquartered entity being added; closes the one state with zero current representation.</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>High-speed catamaran shipbuilding, maritime logistics, allied vessel contracts</t>
+        </is>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="R166" t="n">
+        <v>3</v>
+      </c>
+      <c r="S166" t="n">
+        <v>3</v>
+      </c>
+      <c r="T166" t="n">
+        <v>2</v>
+      </c>
+      <c r="U166" t="n">
+        <v>3</v>
+      </c>
+      <c r="V166" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W166" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X166" t="inlineStr">
+        <is>
+          <t>Fills the Tasmania gap; relevant to maritime logistics and allied vessel procurement news.</t>
+        </is>
+      </c>
+      <c r="Y166" t="inlineStr">
+        <is>
+          <t>Verify current news/press page URL.</t>
+        </is>
+      </c>
+      <c r="Z166" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Liferaft Systems Australia</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Submarine escape, maritime safety systems</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>TAS</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>https://www.liferaftsystems.com/</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>Niche but genuine defence-relevant Tasmanian manufacturer supplying submarine escape systems to allied navies.</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>Submarine escape systems, maritime safety equipment</t>
+        </is>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="R167" t="n">
+        <v>3</v>
+      </c>
+      <c r="S167" t="n">
+        <v>3</v>
+      </c>
+      <c r="T167" t="n">
+        <v>2</v>
+      </c>
+      <c r="U167" t="n">
+        <v>3</v>
+      </c>
+      <c r="V167" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W167" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X167" t="inlineStr">
+        <is>
+          <t>Second Tasmanian entry; relevant to submarine sustainment and allied navy supply relationships.</t>
+        </is>
+      </c>
+      <c r="Y167" t="inlineStr">
+        <is>
+          <t>Verify current news/press page URL.</t>
+        </is>
+      </c>
+      <c r="Z167" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Team Defence Australia</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Export Promotion</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Commonwealth initiative</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>https://www.austrade.gov.au/en/international/team-defence-australia</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>Australian Government</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>Named body for promoting Australian defence exports; no export-promotion source currently exists in the universe.</t>
+        </is>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>Export promotion, trade missions, industry capability showcases</t>
+        </is>
+      </c>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="R168" t="n">
+        <v>4</v>
+      </c>
+      <c r="S168" t="n">
+        <v>3</v>
+      </c>
+      <c r="T168" t="n">
+        <v>2</v>
+      </c>
+      <c r="U168" t="n">
+        <v>3</v>
+      </c>
+      <c r="V168" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W168" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X168" t="inlineStr">
+        <is>
+          <t>Fills export-promotion gap; relevant to capture opportunities criterion in Collection Logic Step 5.</t>
+        </is>
+      </c>
+      <c r="Y168" t="inlineStr">
+        <is>
+          <t>VERIFY current URL - may sit under Austrade or Defence domain.</t>
+        </is>
+      </c>
+      <c r="Z168" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Export Finance Australia</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Adjacent Domain</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Export Finance</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Statutory agency</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>https://www.exportfinance.gov.au/</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>Australian Government</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N169" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>Finances sovereign defence export deals; relevant to capital and contract-financing announcements.</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>Export finance, sovereign defence deal financing</t>
+        </is>
+      </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="R169" t="n">
+        <v>4</v>
+      </c>
+      <c r="S169" t="n">
+        <v>3</v>
+      </c>
+      <c r="T169" t="n">
+        <v>2</v>
+      </c>
+      <c r="U169" t="n">
+        <v>3</v>
+      </c>
+      <c r="V169" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W169" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X169" t="inlineStr">
+        <is>
+          <t>Fills industrial-finance gap adjacent to Defence Industry Development Grants Program.</t>
+        </is>
+      </c>
+      <c r="Z169" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>National Reconstruction Fund Corporation</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Adjacent Domain</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Sovereign Manufacturing</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Statutory agency</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>https://www.nrfc.gov.au/</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>Australian Government</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>Funds sovereign manufacturing capability including defence-adjacent categories; no equivalent source currently tracked.</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>Sovereign manufacturing funding, critical technologies investment</t>
+        </is>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="R170" t="n">
+        <v>4</v>
+      </c>
+      <c r="S170" t="n">
+        <v>3</v>
+      </c>
+      <c r="T170" t="n">
+        <v>2</v>
+      </c>
+      <c r="U170" t="n">
+        <v>3</v>
+      </c>
+      <c r="V170" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W170" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X170" t="inlineStr">
+        <is>
+          <t>Fills industrial-policy funding gap alongside ASCA and the Defence Industry Development Grants Program.</t>
+        </is>
+      </c>
+      <c r="Z170" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>XTEK Limited</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Defence Industry</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Protective equipment, tactical gear</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Listed company channel</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>https://www.xtek.net/</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>XTE</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>ASX-listed defence equipment supplier not currently tracked; relevant to the market-moves section.</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>Protective equipment, tactical and ballistic gear</t>
+        </is>
+      </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="R171" t="n">
+        <v>3</v>
+      </c>
+      <c r="S171" t="n">
+        <v>3</v>
+      </c>
+      <c r="T171" t="n">
+        <v>2</v>
+      </c>
+      <c r="U171" t="n">
+        <v>3</v>
+      </c>
+      <c r="V171" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W171" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X171" t="inlineStr">
+        <is>
+          <t>Closes a specific ASX-listed coverage gap identified during the review.</t>
+        </is>
+      </c>
+      <c r="Y171" t="inlineStr">
+        <is>
+          <t>Verify HQ state and current IR page URL.</t>
+        </is>
+      </c>
+      <c r="Z171" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>AVA Risk Group</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Adjacent Domain</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Fibre-optic sensing, perimeter security</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Listed company channel</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>https://www.avarisk.com/</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>AVA</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>ASX-listed sensing/security company with defence-adjacent applications not currently tracked.</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>Fibre-optic sensing, perimeter and critical infrastructure security</t>
+        </is>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="R172" t="n">
+        <v>3</v>
+      </c>
+      <c r="S172" t="n">
+        <v>3</v>
+      </c>
+      <c r="T172" t="n">
+        <v>2</v>
+      </c>
+      <c r="U172" t="n">
+        <v>3</v>
+      </c>
+      <c r="V172" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W172" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X172" t="inlineStr">
+        <is>
+          <t>Closes a specific ASX-listed coverage gap identified during the review.</t>
+        </is>
+      </c>
+      <c r="Y172" t="inlineStr">
+        <is>
+          <t>Verify HQ state and current IR page URL.</t>
+        </is>
+      </c>
+      <c r="Z172" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Richard Marles X</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Defence</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>VIC</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Minister</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>https://x.com/RichardMarlesMP</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>Faster-breaking parallel channel to an existing LinkedIn/official source.</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>Ministerial and agency statements, breaking commentary</t>
+        </is>
+      </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>Several times weekly</t>
+        </is>
+      </c>
+      <c r="R173" t="n">
+        <v>4</v>
+      </c>
+      <c r="S173" t="n">
+        <v>4</v>
+      </c>
+      <c r="T173" t="n">
+        <v>3</v>
+      </c>
+      <c r="U173" t="n">
+        <v>2</v>
+      </c>
+      <c r="V173" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W173" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X173" t="inlineStr">
+        <is>
+          <t>High-value source for Deputy PM &amp; Minister for Defence statements; X is typically faster than LinkedIn for breaking remarks.</t>
+        </is>
+      </c>
+      <c r="Y173" t="inlineStr">
+        <is>
+          <t>VERIFY HANDLE before activating - not live-confirmed. Mirrors existing LinkedIn entry for the same individual/agency.</t>
+        </is>
+      </c>
+      <c r="Z173" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Pat Conroy X</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Defence</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Minister</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>https://x.com/Pat_ConroyMP</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>Faster-breaking parallel channel to an existing LinkedIn/official source.</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>Ministerial and agency statements, breaking commentary</t>
+        </is>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>Several times weekly</t>
+        </is>
+      </c>
+      <c r="R174" t="n">
+        <v>4</v>
+      </c>
+      <c r="S174" t="n">
+        <v>4</v>
+      </c>
+      <c r="T174" t="n">
+        <v>3</v>
+      </c>
+      <c r="U174" t="n">
+        <v>2</v>
+      </c>
+      <c r="V174" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W174" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X174" t="inlineStr">
+        <is>
+          <t>High-value source for Minister for Defence Industry; parallels existing LinkedIn entry.</t>
+        </is>
+      </c>
+      <c r="Y174" t="inlineStr">
+        <is>
+          <t>VERIFY HANDLE before activating - not live-confirmed. Mirrors existing LinkedIn entry for the same individual/agency.</t>
+        </is>
+      </c>
+      <c r="Z174" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Matt Keogh X</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Defence</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Minister</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>https://x.com/MattKeoghMP</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>Faster-breaking parallel channel to an existing LinkedIn/official source.</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>Ministerial and agency statements, breaking commentary</t>
+        </is>
+      </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>Several times weekly</t>
+        </is>
+      </c>
+      <c r="R175" t="n">
+        <v>4</v>
+      </c>
+      <c r="S175" t="n">
+        <v>4</v>
+      </c>
+      <c r="T175" t="n">
+        <v>3</v>
+      </c>
+      <c r="U175" t="n">
+        <v>2</v>
+      </c>
+      <c r="V175" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W175" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X175" t="inlineStr">
+        <is>
+          <t>Parallels existing LinkedIn entry for Minister for Veterans Affairs and Defence Personnel.</t>
+        </is>
+      </c>
+      <c r="Y175" t="inlineStr">
+        <is>
+          <t>VERIFY HANDLE before activating - not live-confirmed. Mirrors existing LinkedIn entry for the same individual/agency.</t>
+        </is>
+      </c>
+      <c r="Z175" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Defence Australia X</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Defence</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Agency page</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>https://x.com/AusDeptDefence</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>Faster-breaking parallel channel to an existing LinkedIn/official source.</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>Ministerial and agency statements, breaking commentary</t>
+        </is>
+      </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>Several times weekly</t>
+        </is>
+      </c>
+      <c r="R176" t="n">
+        <v>4</v>
+      </c>
+      <c r="S176" t="n">
+        <v>4</v>
+      </c>
+      <c r="T176" t="n">
+        <v>3</v>
+      </c>
+      <c r="U176" t="n">
+        <v>2</v>
+      </c>
+      <c r="V176" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W176" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X176" t="inlineStr">
+        <is>
+          <t>Official Defence channel; typically fastest public channel for breaking statements ahead of press release publication.</t>
+        </is>
+      </c>
+      <c r="Y176" t="inlineStr">
+        <is>
+          <t>VERIFY HANDLE before activating - not live-confirmed. Mirrors existing LinkedIn entry for the same individual/agency.</t>
+        </is>
+      </c>
+      <c r="Z176" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Australian Submarine Agency X</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Defence</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Agency page</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>https://x.com/AusSubmarines</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>Faster-breaking parallel channel to an existing LinkedIn/official source.</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>Ministerial and agency statements, breaking commentary</t>
+        </is>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>Several times weekly</t>
+        </is>
+      </c>
+      <c r="R177" t="n">
+        <v>4</v>
+      </c>
+      <c r="S177" t="n">
+        <v>4</v>
+      </c>
+      <c r="T177" t="n">
+        <v>3</v>
+      </c>
+      <c r="U177" t="n">
+        <v>2</v>
+      </c>
+      <c r="V177" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W177" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X177" t="inlineStr">
+        <is>
+          <t>Parallels existing LinkedIn entry; AUKUS submarine program updates.</t>
+        </is>
+      </c>
+      <c r="Y177" t="inlineStr">
+        <is>
+          <t>VERIFY HANDLE before activating - not live-confirmed. Mirrors existing LinkedIn entry for the same individual/agency.</t>
+        </is>
+      </c>
+      <c r="Z177" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>ASPI / The Strategist X</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Defence</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Think tank publication</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>https://x.com/ASPI_org</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>Faster-breaking parallel channel to an existing LinkedIn/official source.</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>Ministerial and agency statements, breaking commentary</t>
+        </is>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>Several times weekly</t>
+        </is>
+      </c>
+      <c r="R178" t="n">
+        <v>4</v>
+      </c>
+      <c r="S178" t="n">
+        <v>4</v>
+      </c>
+      <c r="T178" t="n">
+        <v>3</v>
+      </c>
+      <c r="U178" t="n">
+        <v>2</v>
+      </c>
+      <c r="V178" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W178" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X178" t="inlineStr">
+        <is>
+          <t>Fast channel for ASPI commentary and report releases ahead of website publication.</t>
+        </is>
+      </c>
+      <c r="Y178" t="inlineStr">
+        <is>
+          <t>VERIFY HANDLE before activating - not live-confirmed. Mirrors existing LinkedIn entry for the same individual/agency.</t>
+        </is>
+      </c>
+      <c r="Z178" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>The Nightly</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Defence</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>National media</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>https://thenightly.com.au/</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>Adds channel diversity (wire service / broadcast / new masthead) without duplicating existing national media.</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>General defence and national security coverage</t>
+        </is>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="R179" t="n">
+        <v>3</v>
+      </c>
+      <c r="S179" t="n">
+        <v>3</v>
+      </c>
+      <c r="T179" t="n">
+        <v>3</v>
+      </c>
+      <c r="U179" t="n">
+        <v>2</v>
+      </c>
+      <c r="V179" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W179" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X179" t="inlineStr">
+        <is>
+          <t>New national digital masthead (Seven West Media); explicitly requested addition.</t>
+        </is>
+      </c>
+      <c r="Y179" t="inlineStr">
+        <is>
+          <t>Verify current defence-specific section/tag URL if one exists.</t>
+        </is>
+      </c>
+      <c r="Z179" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>AAP (Australian Associated Press)</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Defence</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Wire service</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>https://aap.com.au/</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>Adds channel diversity (wire service / broadcast / new masthead) without duplicating existing national media.</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>General defence and national security coverage</t>
+        </is>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="R180" t="n">
+        <v>3</v>
+      </c>
+      <c r="S180" t="n">
+        <v>3</v>
+      </c>
+      <c r="T180" t="n">
+        <v>3</v>
+      </c>
+      <c r="U180" t="n">
+        <v>2</v>
+      </c>
+      <c r="V180" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W180" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X180" t="inlineStr">
+        <is>
+          <t>Primary Australian wire service; often the first point of publication that other outlets republish from.</t>
+        </is>
+      </c>
+      <c r="Y180" t="inlineStr">
+        <is>
+          <t>Verify current defence-specific section/tag URL if one exists.</t>
+        </is>
+      </c>
+      <c r="Z180" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Sky News Australia Defence</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Defence</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Broadcast media</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>https://www.skynews.com.au/</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>Australian</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>Official</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>Adds channel diversity (wire service / broadcast / new masthead) without duplicating existing national media.</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>General defence and national security coverage</t>
+        </is>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="R181" t="n">
+        <v>3</v>
+      </c>
+      <c r="S181" t="n">
+        <v>3</v>
+      </c>
+      <c r="T181" t="n">
+        <v>3</v>
+      </c>
+      <c r="U181" t="n">
+        <v>2</v>
+      </c>
+      <c r="V181" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W181" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X181" t="inlineStr">
+        <is>
+          <t>Only broadcast/TV channel in the universe; adds a channel type not otherwise represented.</t>
+        </is>
+      </c>
+      <c r="Y181" t="inlineStr">
+        <is>
+          <t>Verify current defence-specific section/tag URL if one exists.</t>
+        </is>
+      </c>
+      <c r="Z181" t="inlineStr">
+        <is>
+          <t>NEEDS VERIFICATION</t>
         </is>
       </c>
     </row>
@@ -17940,7 +21315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -18012,6 +21387,18 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>If an item would not change a decision, view or conversation for a partner, deprioritise it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Named exceptions to Australian-headquartered rule</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rule 2 (Australian-headquartered only) excludes offshore-parented company pages by default. Twelve Tier-1 global prime contractors Australian entities (Lockheed Martin Australia, Boeing Defence Australia, BAE Systems Australia, Thales Australia, Rheinmetall Defence Australia, Saab Australia, Elbit Systems of Australia, Leidos Australia, Raytheon Australia, Babcock Australasia, General Dynamics Land Systems - Australia, Naval Group Australia) are named exceptions given their materiality to major contract and sovereign-manufacturing announcements. Any future addition of an offshore-parented entity should be added explicitly to this exception list, not treated as a silent default.</t>
         </is>
       </c>
     </row>

</xml_diff>